<commit_message>
Updated Capture summaries to match Lantows summary data.
</commit_message>
<xml_diff>
--- a/data/Yuma Backwater Stocking and Netting summary.xlsx
+++ b/data/Yuma Backwater Stocking and Netting summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\BackwaterGenetics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE2A5905-828E-4294-855C-E1FFD88D0363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54ADAF0F-9AB5-4E00-86C8-1696B14ECA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{084E9E6E-4555-4D87-9DE7-6AB52ABD8AEB}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{084E9E6E-4555-4D87-9DE7-6AB52ABD8AEB}"/>
   </bookViews>
   <sheets>
     <sheet name="Yuma Cove BW" sheetId="1" r:id="rId1"/>
@@ -600,7 +600,7 @@
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="7.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
     <col min="6" max="6" width="8.140625" customWidth="1"/>
     <col min="7" max="7" width="9.140625" style="4" customWidth="1"/>
     <col min="8" max="8" width="9.28515625" bestFit="1" customWidth="1"/>

</xml_diff>